<commit_message>
migrate csv to json, and add actuators
</commit_message>
<xml_diff>
--- a/dataset/tiny_campus_block/tiny_campus_block.xlsx
+++ b/dataset/tiny_campus_block/tiny_campus_block.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R035cd725788e4ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nodes" sheetId="2" r:id="Rafe60672425b42d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Re1b63112d6ae466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rec70bdf7ffea4d12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nodes" sheetId="2" r:id="R5af3723c39214b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rcd6f888cd692405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuators" sheetId="4" r:id="Rc09588aedfe4499d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -164,7 +165,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -287,6 +288,12 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -338,6 +345,27 @@
     <x:tableColumn id="5" name="walk_time_min"/>
     <x:tableColumn id="6" name="surface_type"/>
     <x:tableColumn id="7" name="accessible"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="CampusActuators" displayName="CampusActuators" ref="A1:M4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="actuator_id"/>
+    <x:tableColumn id="2" name="actuator_type"/>
+    <x:tableColumn id="3" name="anchor_node"/>
+    <x:tableColumn id="4" name="x_m"/>
+    <x:tableColumn id="5" name="y_m"/>
+    <x:tableColumn id="6" name="controlled_edges"/>
+    <x:tableColumn id="7" name="recommended_edges"/>
+    <x:tableColumn id="8" name="cooling_radius_m"/>
+    <x:tableColumn id="9" name="max_heat_reduction_c"/>
+    <x:tableColumn id="10" name="default_wait_time_s"/>
+    <x:tableColumn id="11" name="min_wait_time_s"/>
+    <x:tableColumn id="12" name="max_wait_time_s"/>
+    <x:tableColumn id="13" name="description"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -610,10 +638,10 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="18" t="str">
-        <x:v>Coordinates</x:v>
-      </x:c>
-      <x:c r="B7" s="19" t="str">
-        <x:v>Local x/y coordinates in meters</x:v>
+        <x:v>Actuators</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C7" s="15"/>
       <x:c r="D7" s="15"/>
@@ -622,10 +650,10 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
-        <x:v>Scope</x:v>
+        <x:v>Coordinates and scope</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>One tiny campus block; not a real location</x:v>
+        <x:v>Local x/y coordinates in meters; fictional campus block, not a real location</x:v>
       </x:c>
       <x:c r="C8" s="15"/>
       <x:c r="D8" s="15"/>
@@ -652,7 +680,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="23" t="str">
-        <x:v>Keep node_id and edge_id unique. Every edge endpoint must match a node_id.</x:v>
+        <x:v>Keep node_id, edge_id, and actuator_id unique. Every graph reference must match an existing ID.</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str"/>
       <x:c r="C11" s="23" t="str"/>
@@ -662,7 +690,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="23" t="str">
-        <x:v>The CSV files in the same folder are the canonical machine-readable copies.</x:v>
+        <x:v>The JSON files in the same folder are the canonical machine-readable sources.</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str"/>
       <x:c r="C12" s="23" t="str"/>
@@ -936,7 +964,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c408f3818e849ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd67a18d3841e489c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1284,7 +1312,170 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb899272dfc34712"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4824546a30d64d78"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="21" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="21" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="48" t="str">
+        <x:v>actuator_id</x:v>
+      </x:c>
+      <x:c r="B1" s="48" t="str">
+        <x:v>actuator_type</x:v>
+      </x:c>
+      <x:c r="C1" s="48" t="str">
+        <x:v>anchor_node</x:v>
+      </x:c>
+      <x:c r="D1" s="48" t="str">
+        <x:v>x_m</x:v>
+      </x:c>
+      <x:c r="E1" s="48" t="str">
+        <x:v>y_m</x:v>
+      </x:c>
+      <x:c r="F1" s="48" t="str">
+        <x:v>controlled_edges</x:v>
+      </x:c>
+      <x:c r="G1" s="48" t="str">
+        <x:v>recommended_edges</x:v>
+      </x:c>
+      <x:c r="H1" s="48" t="str">
+        <x:v>cooling_radius_m</x:v>
+      </x:c>
+      <x:c r="I1" s="48" t="str">
+        <x:v>max_heat_reduction_c</x:v>
+      </x:c>
+      <x:c r="J1" s="48" t="str">
+        <x:v>default_wait_time_s</x:v>
+      </x:c>
+      <x:c r="K1" s="48" t="str">
+        <x:v>min_wait_time_s</x:v>
+      </x:c>
+      <x:c r="L1" s="48" t="str">
+        <x:v>max_wait_time_s</x:v>
+      </x:c>
+      <x:c r="M1" s="48" t="str">
+        <x:v>description</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="30" t="str">
+        <x:v>A01</x:v>
+      </x:c>
+      <x:c r="B2" s="30" t="str">
+        <x:v>misting_point</x:v>
+      </x:c>
+      <x:c r="C2" s="30" t="str">
+        <x:v>N08</x:v>
+      </x:c>
+      <x:c r="D2" s="32" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E2" s="32" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F2" s="32"/>
+      <x:c r="G2" s="32"/>
+      <x:c r="H2" s="32" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="I2" s="32" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J2" s="32"/>
+      <x:c r="K2" s="32"/>
+      <x:c r="L2" s="32"/>
+      <x:c r="M2" s="30" t="str">
+        <x:v>Central Green misting point for localized heat reduction</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="30" t="str">
+        <x:v>A02</x:v>
+      </x:c>
+      <x:c r="B3" s="30" t="str">
+        <x:v>traffic_signal</x:v>
+      </x:c>
+      <x:c r="C3" s="30" t="str">
+        <x:v>N09</x:v>
+      </x:c>
+      <x:c r="D3" s="32" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E3" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="32" t="str">
+        <x:v>E07|E08|E12</x:v>
+      </x:c>
+      <x:c r="G3" s="32"/>
+      <x:c r="H3" s="32"/>
+      <x:c r="I3" s="32"/>
+      <x:c r="J3" s="32" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="K3" s="32" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L3" s="32" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="M3" s="30" t="str">
+        <x:v>Adjustable pedestrian signal at the south path intersection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="30" t="str">
+        <x:v>A03</x:v>
+      </x:c>
+      <x:c r="B4" s="30" t="str">
+        <x:v>directional_led</x:v>
+      </x:c>
+      <x:c r="C4" s="30" t="str">
+        <x:v>N02</x:v>
+      </x:c>
+      <x:c r="D4" s="32" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E4" s="32" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F4" s="32"/>
+      <x:c r="G4" s="32" t="str">
+        <x:v>E02|E03|E10</x:v>
+      </x:c>
+      <x:c r="H4" s="32"/>
+      <x:c r="I4" s="32"/>
+      <x:c r="J4" s="32"/>
+      <x:c r="K4" s="32"/>
+      <x:c r="L4" s="32"/>
+      <x:c r="M4" s="30" t="str">
+        <x:v>Directional sign for distributing pedestrian flow from Campus Dining</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a75cc85b62f4125"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
update C to F
</commit_message>
<xml_diff>
--- a/dataset/tiny_campus_block/tiny_campus_block.xlsx
+++ b/dataset/tiny_campus_block/tiny_campus_block.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re18308e3a68848d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nodes" sheetId="2" r:id="Rb53c10da37da4159"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="R9352d01a7ea04be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuators" sheetId="4" r:id="R679ccd8299b3482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6e62470fda224929"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nodes" sheetId="2" r:id="R96e3646e6479469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="3" r:id="Rabfdb42ff22e4ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuators" sheetId="4" r:id="Ra4696048a7824695"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="0&quot;%&quot;"/>
     <x:numFmt numFmtId="203" formatCode="0.00000000"/>
+    <x:numFmt numFmtId="204" formatCode="0.0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -165,7 +166,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="52">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -301,6 +302,7 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -968,7 +970,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e5989a4c35841d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6c87c1d7c96409b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1316,7 +1318,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff5e72f609c4e08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6037355596434f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1363,7 +1365,7 @@
         <x:v>recommended_edges</x:v>
       </x:c>
       <x:c r="H1" s="50" t="str">
-        <x:v>max_heat_reduction_c</x:v>
+        <x:v>max_heat_reduction_f</x:v>
       </x:c>
       <x:c r="I1" s="50" t="str">
         <x:v>default_wait_time_s</x:v>
@@ -1397,8 +1399,8 @@
       </x:c>
       <x:c r="F2" s="3"/>
       <x:c r="G2" s="3"/>
-      <x:c r="H2" s="51" t="n">
-        <x:v>3</x:v>
+      <x:c r="H2" s="52" t="n">
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="I2" s="51"/>
       <x:c r="J2" s="51"/>
@@ -1475,7 +1477,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d0ce7d460b14f65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ddadf6fa1104d08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>